<commit_message>
Write out new version of v0.0.0 treatment & project info tables with selected columns for join in ArcGIS
</commit_message>
<xml_diff>
--- a/data/raw/Project_Info_columns.xlsx
+++ b/data/raw/Project_Info_columns.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eltnmsu-my.sharepoint.com/personal/lossanna_nmsu_edu/Documents/Documents/04_LDC-LTDL/LDC-LTDL/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="215" documentId="8_{48365B36-8811-40C8-A04C-04A62785130B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{52B784EA-D7B9-4CEA-8192-CE99D9BB589B}"/>
+  <xr:revisionPtr revIDLastSave="216" documentId="8_{48365B36-8811-40C8-A04C-04A62785130B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4F04F4DB-1E20-4E1A-867F-ECE8665172C2}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="1620" windowWidth="20376" windowHeight="12096" activeTab="1" xr2:uid="{180FE257-6980-4323-B5A2-AB4BD0017CAE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{180FE257-6980-4323-B5A2-AB4BD0017CAE}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="2" r:id="rId1"/>
@@ -246,9 +246,6 @@
     <t>Monitored_Finish_Year</t>
   </si>
   <si>
-    <t>Year monitoring bega</t>
-  </si>
-  <si>
     <t>Year monitoring ended</t>
   </si>
   <si>
@@ -406,6 +403,9 @@
   </si>
   <si>
     <t>"-1" is yes; "0" is no</t>
+  </si>
+  <si>
+    <t>Year monitoring began</t>
   </si>
 </sst>
 </file>
@@ -829,7 +829,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B6">
         <v>24575</v>
@@ -837,7 +837,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B7">
         <v>50</v>
@@ -1002,7 +1002,7 @@
         <v>34</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
@@ -1016,7 +1016,7 @@
         <v>34</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
@@ -1030,7 +1030,7 @@
         <v>34</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
@@ -1044,7 +1044,7 @@
         <v>34</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
@@ -1058,7 +1058,7 @@
         <v>34</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
@@ -1072,7 +1072,7 @@
         <v>34</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
@@ -1086,7 +1086,7 @@
         <v>34</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
@@ -1100,7 +1100,7 @@
         <v>34</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
@@ -1228,10 +1228,10 @@
         <v>67</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>69</v>
+        <v>122</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
@@ -1239,70 +1239,70 @@
         <v>68</v>
       </c>
       <c r="D29" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="E29" s="4" t="s">
         <v>70</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B30" t="s">
         <v>62</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B31" t="s">
         <v>62</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B32" t="s">
         <v>13</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B33" t="s">
         <v>13</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B34" t="s">
         <v>6</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B35" t="s">
         <v>13</v>
@@ -1316,152 +1316,152 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B36" t="s">
         <v>13</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B37" t="s">
         <v>22</v>
       </c>
       <c r="D37" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E37" s="4" t="s">
         <v>86</v>
-      </c>
-      <c r="E37" s="4" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B38" t="s">
         <v>62</v>
       </c>
       <c r="D38" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E38" s="4" t="s">
         <v>89</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B39" t="s">
         <v>62</v>
       </c>
       <c r="D39" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="E39" s="4" t="s">
         <v>92</v>
-      </c>
-      <c r="E39" s="4" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B40" t="s">
         <v>62</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B41" t="s">
         <v>62</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B42" t="s">
         <v>62</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B43" t="s">
         <v>62</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B44" t="s">
         <v>22</v>
       </c>
       <c r="D44" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="E44" s="4" t="s">
         <v>103</v>
-      </c>
-      <c r="E44" s="4" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B45" t="s">
         <v>6</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B46" t="s">
         <v>22</v>
       </c>
       <c r="C46" t="s">
+        <v>107</v>
+      </c>
+      <c r="D46" s="4" t="s">
         <v>108</v>
-      </c>
-      <c r="D46" s="4" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B47" t="s">
         <v>62</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
@@ -1477,32 +1477,32 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B49" t="s">
         <v>62</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
+        <v>113</v>
+      </c>
+      <c r="B50" t="s">
         <v>114</v>
       </c>
-      <c r="B50" t="s">
+      <c r="D50" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="D50" s="4" t="s">
+      <c r="E50" s="4" t="s">
         <v>116</v>
-      </c>
-      <c r="E50" s="4" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B51" t="s">
         <v>6</v>
@@ -1511,7 +1511,7 @@
         <v>0</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>